<commit_message>
alarmas resueltas, informes periódicos
</commit_message>
<xml_diff>
--- a/reports_output/excel/SunnyApp_Reporte_Alarmas_2026-10-24.xlsx
+++ b/reports_output/excel/SunnyApp_Reporte_Alarmas_2026-10-24.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Reporte de alarmas'!$10:$10</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Reporte de alarmas'!$A$1:$J$21</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Resumen ejecutivo'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Resumen ejecutivo'!$A$1:$H$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm:ss"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,12 +142,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="007F6000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0017365D"/>
       <sz val="10"/>
     </font>
     <font>
@@ -262,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -370,23 +364,17 @@
     <xf numFmtId="0" fontId="17" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -401,7 +389,7 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -528,12 +516,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Resumen ejecutivo'!$A$6:$A$14</f>
+              <f>'Resumen ejecutivo'!$A$6:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Resumen ejecutivo'!$B$6:$B$14</f>
+              <f>'Resumen ejecutivo'!$B$6:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -705,7 +693,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4140000" cy="2700000"/>
@@ -727,7 +715,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4140000" cy="2700000"/>
@@ -1088,7 +1076,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Fecha del reporte: 24/10/2026   |   Generado: 10:36:14   |   Zona horaria: America/Bogota (UTC-05:00)</t>
+          <t>Fecha del reporte: 24/10/2026   |   Generado: 11:31:00   |   Zona horaria: America/Bogota (UTC-05:00)</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1151,12 @@
         <v>0</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>78 d 20 h 51 min  ·  Pérdida de PE</t>
+          <t>78 d 21 h 45 min  ·  Pérdida de PE</t>
         </is>
       </c>
       <c r="I8" s="13" t="n"/>
@@ -1268,12 +1256,12 @@
       </c>
       <c r="I11" s="23" t="inlineStr">
         <is>
-          <t>02 h 49 min</t>
+          <t>03 h 43 min</t>
         </is>
       </c>
       <c r="J11" s="21" t="inlineStr">
         <is>
-          <t>Check Ground Wire</t>
+          <t>Revisar el cable de conexión a tierra.</t>
         </is>
       </c>
     </row>
@@ -1318,12 +1306,12 @@
       </c>
       <c r="I12" s="30" t="inlineStr">
         <is>
-          <t>04 h 43 min</t>
+          <t>05 h 38 min</t>
         </is>
       </c>
       <c r="J12" s="28" t="inlineStr">
         <is>
-          <t>Check CT wiring</t>
+          <t>Revisar el cableado del TC (transformador de corriente).</t>
         </is>
       </c>
     </row>
@@ -1368,12 +1356,12 @@
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>04 h 44 min</t>
+          <t>05 h 38 min</t>
         </is>
       </c>
       <c r="J13" s="21" t="inlineStr">
         <is>
-          <t>Check CT wiring</t>
+          <t>Revisar el cableado del TC (transformador de corriente).</t>
         </is>
       </c>
     </row>
@@ -1418,12 +1406,12 @@
       </c>
       <c r="I14" s="30" t="inlineStr">
         <is>
-          <t>04 h 44 min</t>
+          <t>05 h 39 min</t>
         </is>
       </c>
       <c r="J14" s="28" t="inlineStr">
         <is>
-          <t>Check CT wiring</t>
+          <t>Revisar el cableado del TC (transformador de corriente).</t>
         </is>
       </c>
     </row>
@@ -1468,12 +1456,12 @@
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>04 h 45 min</t>
+          <t>05 h 40 min</t>
         </is>
       </c>
       <c r="J15" s="21" t="inlineStr">
         <is>
-          <t>Check CT wiring</t>
+          <t>Revisar el cableado del TC (transformador de corriente).</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1506,12 @@
       </c>
       <c r="I16" s="33" t="inlineStr">
         <is>
-          <t>7 d 23 h 20 min</t>
+          <t>8 d 00 h 15 min</t>
         </is>
       </c>
       <c r="J16" s="28" t="inlineStr">
         <is>
-          <t>Check Ground Wire</t>
+          <t>Revisar el cable de conexión a tierra.</t>
         </is>
       </c>
     </row>
@@ -1563,18 +1551,17 @@
       </c>
       <c r="H17" s="39" t="inlineStr">
         <is>
-          <t>Persistente</t>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="I17" s="33" t="inlineStr">
         <is>
-          <t>20 d 19 h 26 min</t>
+          <t>20 d 20 h 20 min</t>
         </is>
       </c>
       <c r="J17" s="35" t="inlineStr">
         <is>
-          <t>1. The alarm goes away when the grid comes back up.
-2. Check if the AC wiring or the switch is disconnected.</t>
+          <t>1. La alarma desaparece cuando regresa la energía de la red. 2. Revisar si el cableado AC o el interruptor está desconectado.</t>
         </is>
       </c>
     </row>
@@ -1612,19 +1599,19 @@
           <t>Ocurriendo</t>
         </is>
       </c>
-      <c r="H18" s="40" t="inlineStr">
-        <is>
-          <t>Persistente</t>
+      <c r="H18" s="32" t="inlineStr">
+        <is>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="I18" s="33" t="inlineStr">
         <is>
-          <t>29 d 08 h 48 min</t>
+          <t>29 d 09 h 43 min</t>
         </is>
       </c>
       <c r="J18" s="28" t="inlineStr">
         <is>
-          <t>Check Ground Wire</t>
+          <t>Revisar el cable de conexión a tierra.</t>
         </is>
       </c>
     </row>
@@ -1662,19 +1649,19 @@
           <t>Ocurriendo</t>
         </is>
       </c>
-      <c r="H19" s="41" t="inlineStr">
-        <is>
-          <t>Persistente</t>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="I19" s="33" t="inlineStr">
         <is>
-          <t>61 d 20 h 25 min</t>
+          <t>61 d 21 h 19 min</t>
         </is>
       </c>
       <c r="J19" s="21" t="inlineStr">
         <is>
-          <t>Check Ground Wire</t>
+          <t>Revisar el cable de conexión a tierra.</t>
         </is>
       </c>
     </row>
@@ -1712,19 +1699,19 @@
           <t>Ocurriendo</t>
         </is>
       </c>
-      <c r="H20" s="40" t="inlineStr">
-        <is>
-          <t>Persistente</t>
+      <c r="H20" s="32" t="inlineStr">
+        <is>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="I20" s="33" t="inlineStr">
         <is>
-          <t>78 d 19 h 50 min</t>
+          <t>78 d 20 h 44 min</t>
         </is>
       </c>
       <c r="J20" s="28" t="inlineStr">
         <is>
-          <t>Check CT wiring</t>
+          <t>Revisar el cableado del TC (transformador de corriente).</t>
         </is>
       </c>
     </row>
@@ -1762,19 +1749,19 @@
           <t>Ocurriendo</t>
         </is>
       </c>
-      <c r="H21" s="41" t="inlineStr">
-        <is>
-          <t>Persistente</t>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="I21" s="33" t="inlineStr">
         <is>
-          <t>78 d 20 h 51 min</t>
+          <t>78 d 21 h 45 min</t>
         </is>
       </c>
       <c r="J21" s="21" t="inlineStr">
         <is>
-          <t>Check Ground Wire</t>
+          <t>Revisar el cable de conexión a tierra.</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1829,403 +1816,385 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>SUNNY APP  |  RESUMEN EJECUTIVO DE ALARMAS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="43" t="inlineStr">
-        <is>
-          <t>Plataforma GoodWe  ·  24/10/2026 10:36 (America/Bogota)</t>
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>Plataforma GoodWe  ·  24/10/2026 11:31 (America/Bogota)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Alarmas activas por planta (top 10)</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="42" t="inlineStr">
         <is>
           <t>Distribución por tipo de alarma</t>
         </is>
       </c>
-      <c r="G4" s="44" t="inlineStr">
+      <c r="G4" s="42" t="inlineStr">
         <is>
           <t>Distribución por estado</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="45" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>Planta</t>
         </is>
       </c>
-      <c r="B5" s="45" t="inlineStr">
+      <c r="B5" s="43" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D5" s="45" t="inlineStr">
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E5" s="45" t="inlineStr">
+      <c r="E5" s="43" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="G5" s="45" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t>Estado · situación</t>
         </is>
       </c>
-      <c r="H5" s="45" t="inlineStr">
+      <c r="H5" s="43" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>507. ABDERRAMAN MARTÍNEZ (16,94 kWp - 62 kWh)</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="46" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>Información de condición de operación</t>
         </is>
       </c>
-      <c r="E6" s="47" t="n">
+      <c r="E6" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="46" t="inlineStr">
+      <c r="G6" s="44" t="inlineStr">
         <is>
           <t>Ocurriendo · Nueva</t>
         </is>
       </c>
-      <c r="H6" s="47" t="n">
-        <v>6</v>
+      <c r="H6" s="45" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>600. GRANJA PRODUCTORA (7,56 kWp - 30 kWh)</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="46" t="inlineStr">
+        <is>
+          <t>Eventos de protección</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>527. FRANCISCO GARCÍA (13,86 kWp - 51 kWh)</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B8" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>Eventos de protección</t>
-        </is>
-      </c>
-      <c r="E7" s="49" t="n">
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>482. ROCIO CUPITRE PIMENTONIS (11,16 kWp - 42 kWh)</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="48" t="inlineStr">
-        <is>
-          <t>Ocurriendo · Persistente</t>
-        </is>
-      </c>
-      <c r="H7" s="49" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="46" t="inlineStr">
-        <is>
-          <t>482. ROCIO CUPITRE PIMENTONIS (11,16 kWp - 42 kWh)</t>
-        </is>
-      </c>
-      <c r="B8" s="47" t="n">
+    </row>
+    <row r="10">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>Villa Valentina</t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="48" t="inlineStr">
-        <is>
-          <t>Villa Valentina</t>
-        </is>
-      </c>
-      <c r="B9" s="49" t="n">
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>Patricia Ninco Caguan</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>Patricia Ninco Caguan</t>
-        </is>
-      </c>
-      <c r="B10" s="47" t="n">
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>625. Coorporación universiteria del huila, corhuil</t>
+        </is>
+      </c>
+      <c r="B12" s="45" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>601 Ramiro Núñez</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="48" t="inlineStr">
+        <is>
+          <t>Alarmas activas más antiguas (top 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>Planta</t>
+        </is>
+      </c>
+      <c r="B33" s="43" t="inlineStr">
+        <is>
+          <t>Duración</t>
+        </is>
+      </c>
+      <c r="D33" s="43" t="inlineStr">
+        <is>
+          <t>Alarma</t>
+        </is>
+      </c>
+      <c r="E33" s="43" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="G33" s="43" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>600 Granja Productora</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="inlineStr">
+        <is>
+          <t>78 d 21 h 45 min</t>
+        </is>
+      </c>
+      <c r="D34" s="50" t="inlineStr">
+        <is>
+          <t>Pérdida de PE</t>
+        </is>
+      </c>
+      <c r="E34" s="50" t="inlineStr">
+        <is>
+          <t>Inversor 1</t>
+        </is>
+      </c>
+      <c r="G34" s="50" t="inlineStr">
+        <is>
+          <t>56000NBB262L0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>600. GRANJA PRODUCTORA (7,56 kWp - 30 kWh)</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="inlineStr">
+        <is>
+          <t>78 d 20 h 44 min</t>
+        </is>
+      </c>
+      <c r="D35" s="50" t="inlineStr">
+        <is>
+          <t>Pérdida de TC</t>
+        </is>
+      </c>
+      <c r="E35" s="50" t="inlineStr">
+        <is>
+          <t>Inversor 1</t>
+        </is>
+      </c>
+      <c r="G35" s="50" t="inlineStr">
+        <is>
+          <t>56000NBB262L0005</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>601 Ramiro Núñez</t>
+        </is>
+      </c>
+      <c r="B36" s="50" t="inlineStr">
+        <is>
+          <t>61 d 21 h 19 min</t>
+        </is>
+      </c>
+      <c r="D36" s="50" t="inlineStr">
+        <is>
+          <t>Pérdida de PE</t>
+        </is>
+      </c>
+      <c r="E36" s="50" t="inlineStr">
+        <is>
+          <t>Inversor 2</t>
+        </is>
+      </c>
+      <c r="G36" s="50" t="inlineStr">
+        <is>
+          <t>56000NBB262L0047</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>507. ABDERRAMAN MARTÍNEZ (16,94 kWp - 62 kWh)</t>
+        </is>
+      </c>
+      <c r="B37" s="50" t="inlineStr">
+        <is>
+          <t>29 d 09 h 43 min</t>
+        </is>
+      </c>
+      <c r="D37" s="50" t="inlineStr">
+        <is>
+          <t>Pérdida de PE</t>
+        </is>
+      </c>
+      <c r="E37" s="50" t="inlineStr">
+        <is>
+          <t>Inversor 2</t>
+        </is>
+      </c>
+      <c r="G37" s="50" t="inlineStr">
+        <is>
+          <t>56000NBB25AL0077</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="49" t="inlineStr">
         <is>
           <t>625. Coorporación universiteria del huila, corhuil</t>
         </is>
       </c>
-      <c r="B11" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t>601 Ramiro Núñez</t>
-        </is>
-      </c>
-      <c r="B12" s="47" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="48" t="inlineStr">
-        <is>
-          <t>600. GRANJA PRODUCTORA (7,56 kWp - 30 kWh)</t>
-        </is>
-      </c>
-      <c r="B13" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="46" t="inlineStr">
-        <is>
-          <t>600 Granja Productora</t>
-        </is>
-      </c>
-      <c r="B14" s="47" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="50" t="inlineStr">
-        <is>
-          <t>Alarmas activas más antiguas (top 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="45" t="inlineStr">
-        <is>
-          <t>Planta</t>
-        </is>
-      </c>
-      <c r="B34" s="45" t="inlineStr">
-        <is>
-          <t>Duración</t>
-        </is>
-      </c>
-      <c r="D34" s="45" t="inlineStr">
-        <is>
-          <t>Alarma</t>
-        </is>
-      </c>
-      <c r="E34" s="45" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="G34" s="45" t="inlineStr">
-        <is>
-          <t>SN</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="51" t="inlineStr">
-        <is>
-          <t>600 Granja Productora</t>
-        </is>
-      </c>
-      <c r="B35" s="52" t="inlineStr">
-        <is>
-          <t>78 d 20 h 51 min</t>
-        </is>
-      </c>
-      <c r="D35" s="52" t="inlineStr">
-        <is>
-          <t>Pérdida de PE</t>
-        </is>
-      </c>
-      <c r="E35" s="52" t="inlineStr">
+      <c r="B38" s="50" t="inlineStr">
+        <is>
+          <t>20 d 20 h 20 min</t>
+        </is>
+      </c>
+      <c r="D38" s="50" t="inlineStr">
+        <is>
+          <t>Corte de energía de la red</t>
+        </is>
+      </c>
+      <c r="E38" s="50" t="inlineStr">
         <is>
           <t>Inversor 1</t>
         </is>
       </c>
-      <c r="G35" s="52" t="inlineStr">
-        <is>
-          <t>56000NBB262L0005</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="51" t="inlineStr">
-        <is>
-          <t>600. GRANJA PRODUCTORA (7,56 kWp - 30 kWh)</t>
-        </is>
-      </c>
-      <c r="B36" s="52" t="inlineStr">
-        <is>
-          <t>78 d 19 h 50 min</t>
-        </is>
-      </c>
-      <c r="D36" s="52" t="inlineStr">
-        <is>
-          <t>Pérdida de TC</t>
-        </is>
-      </c>
-      <c r="E36" s="52" t="inlineStr">
-        <is>
-          <t>Inversor 1</t>
-        </is>
-      </c>
-      <c r="G36" s="52" t="inlineStr">
-        <is>
-          <t>56000NBB262L0005</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="51" t="inlineStr">
-        <is>
-          <t>601 Ramiro Núñez</t>
-        </is>
-      </c>
-      <c r="B37" s="52" t="inlineStr">
-        <is>
-          <t>61 d 20 h 25 min</t>
-        </is>
-      </c>
-      <c r="D37" s="52" t="inlineStr">
-        <is>
-          <t>Pérdida de PE</t>
-        </is>
-      </c>
-      <c r="E37" s="52" t="inlineStr">
-        <is>
-          <t>Inversor 2</t>
-        </is>
-      </c>
-      <c r="G37" s="52" t="inlineStr">
-        <is>
-          <t>56000NBB262L0047</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="51" t="inlineStr">
-        <is>
-          <t>507. ABDERRAMAN MARTÍNEZ (16,94 kWp - 62 kWh)</t>
-        </is>
-      </c>
-      <c r="B38" s="52" t="inlineStr">
-        <is>
-          <t>29 d 08 h 48 min</t>
-        </is>
-      </c>
-      <c r="D38" s="52" t="inlineStr">
-        <is>
-          <t>Pérdida de PE</t>
-        </is>
-      </c>
-      <c r="E38" s="52" t="inlineStr">
-        <is>
-          <t>Inversor 2</t>
-        </is>
-      </c>
-      <c r="G38" s="52" t="inlineStr">
-        <is>
-          <t>56000NBB25AL0077</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="51" t="inlineStr">
-        <is>
-          <t>625. Coorporación universiteria del huila, corhuil</t>
-        </is>
-      </c>
-      <c r="B39" s="52" t="inlineStr">
-        <is>
-          <t>20 d 19 h 26 min</t>
-        </is>
-      </c>
-      <c r="D39" s="52" t="inlineStr">
-        <is>
-          <t>Corte de energía de la red</t>
-        </is>
-      </c>
-      <c r="E39" s="52" t="inlineStr">
-        <is>
-          <t>Inversor 1</t>
-        </is>
-      </c>
-      <c r="G39" s="52" t="inlineStr">
+      <c r="G38" s="50" t="inlineStr">
         <is>
           <t>5017KDTR257L0023</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="50" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="48" t="inlineStr">
         <is>
           <t>Cómo leer este resumen</t>
         </is>
       </c>
     </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="51" t="inlineStr">
+        <is>
+          <t>•  Es una foto de las alarmas que estaban activas en la plataforma GoodWe en el momento de la lectura.</t>
+        </is>
+      </c>
+    </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="53" t="inlineStr">
-        <is>
-          <t>•  Es una foto de las alarmas que estaban activas en la plataforma GoodWe en el momento de la lectura.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="53" t="inlineStr">
+      <c r="A42" s="51" t="inlineStr">
         <is>
           <t>•  Por planta: muestra dónde se concentran las alarmas. Una planta con varias alarmas debe revisarse primero.</t>
         </is>
       </c>
     </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="51" t="inlineStr">
+        <is>
+          <t>•  Por tipo: los "Eventos de protección" suelen requerir atención más rápida. La "Información de condición de operación" son avisos del equipo (por ejemplo, pérdida de PE o de TC) que el equipo técnico debe validar en sitio; no confirman por sí solos un daño físico.</t>
+        </is>
+      </c>
+    </row>
     <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="53" t="inlineStr">
-        <is>
-          <t>•  Por tipo: los "Eventos de protección" suelen requerir atención más rápida. La "Información de condición de operación" son avisos del equipo (por ejemplo, pérdida de PE o de TC) que el equipo técnico debe validar en sitio; no confirman por sí solos un daño físico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="40" customHeight="1">
-      <c r="A45" s="53" t="inlineStr">
+      <c r="A44" s="51" t="inlineStr">
         <is>
           <t>•  Nueva / Persistente: "Nueva" significa que el sistema la detectó por primera vez hoy; "Persistente", que ya venía de lecturas anteriores. No indica cuándo empezó la alarma: eso lo dice la columna Duración.</t>
         </is>
       </c>
     </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="51" t="inlineStr">
+        <is>
+          <t>•  Alarmas más antiguas: llevan más tiempo sin resolverse; son la prioridad de seguimiento.</t>
+        </is>
+      </c>
+    </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="53" t="inlineStr">
-        <is>
-          <t>•  Alarmas más antiguas: llevan más tiempo sin resolverse; son la prioridad de seguimiento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="53" t="inlineStr">
+      <c r="A46" s="51" t="inlineStr">
         <is>
           <t>•  Las alarmas resueltas salen automáticamente del reporte y no se muestran aquí.</t>
         </is>
@@ -2238,11 +2207,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A47:H47"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.5" footer="0.5"/>

</xml_diff>